<commit_message>
feat: implement TemplateModal and LivePreview components with custom Tailwind styles
</commit_message>
<xml_diff>
--- a/Test_Apparel_Business_Zone.xlsx
+++ b/Test_Apparel_Business_Zone.xlsx
@@ -1,41 +1,119 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr codeName="ThisWorkbook"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vj\IdeaProjects\WAReachApparel\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB8429DD-3F42-4437-A0DF-342D1C29A389}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
     <sheet name="WA-Download Group Phone Numbers" sheetId="1" r:id="rId1"/>
   </sheets>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
-  <metadataTypes count="1">
-    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLDAPR" count="1">
-    <bk>
-      <extLst>
-        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
-          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <cellMetadata count="1">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-  </cellMetadata>
-</metadata>
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="29">
+  <si>
+    <t>Country Code</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Phone Number 			</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Saved Name 					</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Public Display Name 					</t>
+  </si>
+  <si>
+    <t>Is Admin?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Group_Name 					</t>
+  </si>
+  <si>
+    <t>+91</t>
+  </si>
+  <si>
+    <t>918310438481</t>
+  </si>
+  <si>
+    <t>Abdul Buyer</t>
+  </si>
+  <si>
+    <t>Abdul</t>
+  </si>
+  <si>
+    <t>Apparel Business Zone 🌹</t>
+  </si>
+  <si>
+    <t>Anand Fab Distributors Buyer</t>
+  </si>
+  <si>
+    <t>Ananda V</t>
+  </si>
+  <si>
+    <t>ARULALAN PILLAI</t>
+  </si>
+  <si>
+    <t>R.ARULALAN  PILLAI</t>
+  </si>
+  <si>
+    <t>Aseem Chitkara Buyer</t>
+  </si>
+  <si>
+    <t>Aseem Chitkara</t>
+  </si>
+  <si>
+    <t>ASIM Kurti Buyer</t>
+  </si>
+  <si>
+    <t>ASIM</t>
+  </si>
+  <si>
+    <t>Brijesh Shah Buyer</t>
+  </si>
+  <si>
+    <t>Brijesh Shah</t>
+  </si>
+  <si>
+    <t>Harsha Hindhupur</t>
+  </si>
+  <si>
+    <t>Shree</t>
+  </si>
+  <si>
+    <t>Hegde Buyer</t>
+  </si>
+  <si>
+    <t>Kattanai Md Nizamudeen Buyer</t>
+  </si>
+  <si>
+    <t>Kattanai Md Nizamudeen J</t>
+  </si>
+  <si>
+    <t>kavshik Buyer</t>
+  </si>
+  <si>
+    <t>Only limited rows are available as you are using Free Version. Subscribe now to get full list</t>
+  </si>
+  <si>
+    <t>Vijay Pradhan</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="1">
-    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
-  </numFmts>
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -65,13 +143,21 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -396,240 +482,245 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F12"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="3" max="3" width="28.19921875" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Country Code</v>
-      </c>
-      <c r="B1" t="str">
-        <v xml:space="preserve">Phone Number 			</v>
-      </c>
-      <c r="C1" t="str">
-        <v xml:space="preserve">Saved Name 					</v>
-      </c>
-      <c r="D1" t="str">
-        <v xml:space="preserve">Public Display Name 					</v>
-      </c>
-      <c r="E1" t="str">
-        <v>Is Admin?</v>
-      </c>
-      <c r="F1" t="str">
-        <v xml:space="preserve">Group_Name 					</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>+91</v>
-      </c>
-      <c r="B2" t="str">
-        <v>918310438481</v>
-      </c>
-      <c r="C2" t="str">
-        <v>Abdul Buyer</v>
-      </c>
-      <c r="D2" t="str">
-        <v>Abdul</v>
+    <row r="1" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2" t="s">
+        <v>9</v>
       </c>
       <c r="E2" t="b">
         <v>0</v>
       </c>
-      <c r="F2" t="str">
-        <v>Apparel Business Zone 🌹</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>+91</v>
-      </c>
-      <c r="B3" t="str">
-        <v>918310438481</v>
-      </c>
-      <c r="C3" t="str">
-        <v>Anand Fab Distributors Buyer</v>
-      </c>
-      <c r="D3" t="str">
-        <v>Ananda V</v>
+      <c r="F2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" t="s">
+        <v>12</v>
       </c>
       <c r="E3" t="b">
         <v>0</v>
       </c>
-      <c r="F3" t="str">
-        <v>Apparel Business Zone 🌹</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>+91</v>
-      </c>
-      <c r="B4" t="str">
-        <v>918310438481</v>
-      </c>
-      <c r="C4" t="str">
-        <v>ARULALAN PILLAI</v>
-      </c>
-      <c r="D4" t="str">
-        <v>R.ARULALAN  PILLAI</v>
+      <c r="F3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4" t="s">
+        <v>14</v>
       </c>
       <c r="E4" t="b">
         <v>0</v>
       </c>
-      <c r="F4" t="str">
-        <v>Apparel Business Zone 🌹</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>+91</v>
-      </c>
-      <c r="B5" t="str">
-        <v>918310438481</v>
-      </c>
-      <c r="C5" t="str">
-        <v>Aseem Chitkara Buyer</v>
-      </c>
-      <c r="D5" t="str">
-        <v>Aseem Chitkara</v>
+      <c r="F4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" t="s">
+        <v>15</v>
+      </c>
+      <c r="D5" t="s">
+        <v>16</v>
       </c>
       <c r="E5" t="b">
         <v>0</v>
       </c>
-      <c r="F5" t="str">
-        <v>Apparel Business Zone 🌹</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>+91</v>
-      </c>
-      <c r="B6" t="str">
-        <v>918310438481</v>
-      </c>
-      <c r="C6" t="str">
-        <v>ASIM Kurti Buyer</v>
-      </c>
-      <c r="D6" t="str">
-        <v>ASIM</v>
+      <c r="F5" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C6" t="s">
+        <v>17</v>
+      </c>
+      <c r="D6" t="s">
+        <v>18</v>
       </c>
       <c r="E6" t="b">
         <v>0</v>
       </c>
-      <c r="F6" t="str">
-        <v>Apparel Business Zone 🌹</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>+91</v>
-      </c>
-      <c r="B7" t="str">
-        <v>918310438481</v>
-      </c>
-      <c r="C7" t="str">
-        <v>Brijesh Shah Buyer</v>
-      </c>
-      <c r="D7" t="str">
-        <v>Brijesh Shah</v>
+      <c r="F6" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C7" t="s">
+        <v>19</v>
+      </c>
+      <c r="D7" t="s">
+        <v>20</v>
       </c>
       <c r="E7" t="b">
         <v>0</v>
       </c>
-      <c r="F7" t="str">
-        <v>Apparel Business Zone 🌹</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>+91</v>
-      </c>
-      <c r="B8" t="str">
-        <v>918310438481</v>
-      </c>
-      <c r="C8" t="str">
-        <v>Harsha Hindhupur</v>
-      </c>
-      <c r="D8" t="str">
-        <v>Shree</v>
+      <c r="F7" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>6</v>
+      </c>
+      <c r="B8" t="s">
+        <v>7</v>
+      </c>
+      <c r="C8" t="s">
+        <v>21</v>
+      </c>
+      <c r="D8" t="s">
+        <v>22</v>
       </c>
       <c r="E8" t="b">
         <v>0</v>
       </c>
-      <c r="F8" t="str">
-        <v>Apparel Business Zone 🌹</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>+91</v>
-      </c>
-      <c r="B9" t="str">
-        <v>918310438481</v>
-      </c>
-      <c r="C9" t="str">
-        <v>Hegde Buyer</v>
-      </c>
-      <c r="D9" t="str">
-        <v>Hegde Buyer</v>
+      <c r="F8" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>6</v>
+      </c>
+      <c r="B9" t="s">
+        <v>7</v>
+      </c>
+      <c r="C9" t="s">
+        <v>23</v>
+      </c>
+      <c r="D9" t="s">
+        <v>23</v>
       </c>
       <c r="E9" t="b">
         <v>0</v>
       </c>
-      <c r="F9" t="str">
-        <v>Apparel Business Zone 🌹</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>+91</v>
-      </c>
-      <c r="B10" t="str">
-        <v>918310438481</v>
-      </c>
-      <c r="C10" t="str">
-        <v>Kattanai Md Nizamudeen Buyer</v>
-      </c>
-      <c r="D10" t="str">
-        <v>Kattanai Md Nizamudeen J</v>
+      <c r="F9" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>6</v>
+      </c>
+      <c r="B10" t="s">
+        <v>7</v>
+      </c>
+      <c r="C10" t="s">
+        <v>24</v>
+      </c>
+      <c r="D10" t="s">
+        <v>25</v>
       </c>
       <c r="E10" t="b">
         <v>0</v>
       </c>
-      <c r="F10" t="str">
-        <v>Apparel Business Zone 🌹</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v>+91</v>
-      </c>
-      <c r="B11" t="str">
-        <v>918310438481</v>
-      </c>
-      <c r="C11" t="str">
-        <v>kavshik Buyer</v>
-      </c>
-      <c r="D11" t="str">
-        <v>kavshik</v>
+      <c r="F10" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>6</v>
+      </c>
+      <c r="B11" t="s">
+        <v>7</v>
+      </c>
+      <c r="C11" t="s">
+        <v>26</v>
+      </c>
+      <c r="D11" t="s">
+        <v>28</v>
       </c>
       <c r="E11" t="b">
         <v>0</v>
       </c>
-      <c r="F11" t="str">
-        <v>Apparel Business Zone 🌹</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="str">
-        <v>Only limited rows are available as you are using Free Version. Subscribe now to get full list</v>
-      </c>
-      <c r="B12" t="str">
-        <v>918310438481</v>
+      <c r="F11" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>27</v>
+      </c>
+      <c r="B12" t="s">
+        <v>7</v>
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F12"/>
+    <ignoredError sqref="A1:F10 A12:F12 A11:C11 E11:F11" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>